<commit_message>
refactor: v2.0.0 generalize to discrete manufacturing
</commit_message>
<xml_diff>
--- a/02-精益培训/03-培训计划/01-年度培训计划模板.xlsx
+++ b/02-精益培训/03-培训计划/01-年度培训计划模板.xlsx
@@ -90,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -117,11 +117,20 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="001F3A5F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -145,6 +154,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -528,7 +538,13 @@
           <t>01-年度培训计划模板</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="11" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -536,6 +552,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -543,6 +560,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
@@ -550,6 +568,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -557,6 +576,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
@@ -564,6 +584,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -571,6 +592,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -578,13 +600,15 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>以下为某金属紧固件企业第一年精益培训的年度安排示例：</t>
-        </is>
-      </c>
-    </row>
+          <t>以下为某金属制造企业第一年精益培训的年度安排示例：</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
@@ -592,6 +616,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -599,6 +624,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
@@ -606,6 +632,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
@@ -613,6 +640,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
@@ -620,6 +648,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
@@ -655,6 +684,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
@@ -662,6 +692,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
@@ -697,6 +728,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
@@ -704,6 +736,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>

</xml_diff>